<commit_message>
Update detection coverage matrix based on divynahsu feedback and gap analysis fixes
</commit_message>
<xml_diff>
--- a/important_files/detection_coverage_matrix_final.xlsx
+++ b/important_files/detection_coverage_matrix_final.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Coverage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,20 +427,6 @@
   </sheetPr>
   <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -562,7 +548,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -594,7 +580,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Partial: We have strong behavioral detection rules (process chains), but Sigma cannot perform real-time blocking.</t>
+          <t>Strong behavioral detection capability through stateful streaming correlation including process chains, parent-child relationships, temporal sequences, threshold detection, aggregation, cross-sensor correlation, attack graph reasoning and behavioral validation. Real-time prevention/blocking is outside the detection engine and requires an EDR agent.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -748,7 +734,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -775,7 +761,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1612,7 +1598,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1749,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Gap: DGA and beacon detection are statistical/ML problems, making Sigma rules weak even with logs.</t>
+          <t>Supports behavioral beacon detection, periodic communication analysis, prevalence-based detection, cross-sensor correlation and attack graph reasoning using Zeek, Suricata and endpoint telemetry. Full DGA classification, encrypted HTTPS payload inspection, TLS fingerprinting and ML-based beacon analytics require NDR or specialized analytics.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1892,7 +1878,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Gap: Sysmon Event ID 3 only logs IP/Port. It cannot perform deep packet inspection, protocol anomalies, or IoT visibility.</t>
+          <t>Strong detection using Zeek, Suricata, network flow correlation, attack graph reasoning, cross-sensor joins, prevalence analysis and behavioral analytics. Deep packet inspection, protocol decoding, IoT discovery and advanced NDR analytics require dedicated NDR platforms.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2046,7 +2032,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2094,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2156,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix row 5 Gap Type and Tooling flag inconsistency
</commit_message>
<xml_diff>
--- a/important_files/detection_coverage_matrix_final.xlsx
+++ b/important_files/detection_coverage_matrix_final.xlsx
@@ -724,12 +724,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Fully Covered</t>
+          <t>Tooling / Capability Gap</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">

</xml_diff>

<commit_message>
chore: clean up temporary scripts and update detection matrix with accurate SOAR terminology
</commit_message>
<xml_diff>
--- a/important_files/detection_coverage_matrix_final.xlsx
+++ b/important_files/detection_coverage_matrix_final.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Real-time prevention and pre-execution ML scoring are architectural capabilities that require a dedicated NGAV/EDR agent on the endpoint. Our detection engine operates post-execution on telemetry and cannot perform this point-in-time stateless prevention.</t>
+          <t>Real-time prevention and pre-execution ML scoring are architectural capabilities that require a dedicated NGAV/EDR agent on the endpoint. Our SIEM detection engine analyzes logs after an event has occurred. It cannot perform instantaneous file scanning or immediate blocking before execution (which is what traditional Antivirus does).</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial (Detection Only)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Strong behavioral detection capability through stateful streaming correlation is fully covered by 470+ active correlation rules (e.g., AN0827-T1561.002-DET0297, AN0602-T1486-DET0215). Real-time prevention/blocking is out of scope. We lack the advanced EDR integration required for process termination or active prevention.</t>
+          <t>Strong behavioral detection capability is fully covered by 470+ active correlation rules. The engine tracks sequences of events over short time windows (e.g., detecting if Event A is followed by Event B within 5 minutes) (e.g., AN0827-T1561.002-DET0297, AN0602-T1486-DET0215). Real-time prevention/blocking is out of scope as it requires an EDR agent. Real-time response requires complex API integrations which our current SOAR cannot perform.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Yes, via SOAR playbook calling EDR API.</t>
+          <t>No. Our current SOAR cannot perform complex API integrations.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SOAR playbook: take-response-action via EDR API</t>
+          <t>Advanced SOAR / API Integration</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,12 +605,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Process Hollowing detection is covered (rule AN1076-T1055.012-DET0382). However, we have significant gaps for the other techniques: To detect LOLBAS, we need Sysmon Event ID 1. To detect hidden scripts via AMSI, we need Windows Event 1116/1117. For Windows to generate these logs, IT must enable Script Block Logging via Group Policy (GPO). Detecting Reflective DLL and real-time blocking are out of scope.</t>
+          <t>Process Hollowing detection is covered (rule AN1076-T1055.012-DET0382). However, we have significant gaps for the other techniques: To detect LOLBAS (hackers abusing built-in Windows tools), we need Sysmon Event ID 1 to see the exact tool name (OriginalFileName) and what command was typed (CommandLine). To detect hidden scripts via AMSI, we need Windows Event 1116/1117 to read the actual script content (ScriptBlockText). For Windows to even generate these logs, IT must first enable 'Script Block Logging' via Group Policy (GPO). Finally, detecting Reflective DLL (which hides directly in RAM) and real-time blocking are out of scope. SIEM only reads logs; scanning RAM and blocking attacks requires a dedicated EDR agent. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Rule</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -699,12 +699,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial (Detection Only)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Full endpoint host isolation via EDR is out of scope. However, network containment can be achieved via SOAR IP/firewall blocking. The SIEM detects the condition, and a SOAR playbook executes firewall blocking.</t>
+          <t>While we can audit when a hacker tampers with a host firewall, performing actual one-click network containment and remote site isolation are active response capabilities. This requires a dedicated EDR agent. Our SIEM correlation engine operates passively on logs and cannot perform this physical containment function. Note: While our current SOAR is capable of simple tasks like perimeter IP blocking and basic firewall rules, full endpoint isolation requires complex EDR API integrations which it cannot currently perform.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Yes, via SOAR playbook calling EDR API.</t>
+          <t>No. Our current SOAR cannot perform complex API integrations.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>SOAR playbook: Firewall/IP blocking</t>
+          <t>Advanced SOAR / API Integration</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -729,12 +729,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Out of Scope</t>
+          <t>Partial (Detection Only)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>A SIEM is a passive log analytics tool; it cannot perform active live response or remote remediation on endpoints (like killing processes or isolating machines). We lack the advanced EDR integration required to perform these actions.</t>
+          <t>A SIEM is a passive log analytics tool; it cannot perform active 'live response' or 'remote remediation' on endpoints (like killing processes or isolating machines). This capability physically requires an EDR agent. Real-time response requires complex API integrations which our current SOAR cannot perform.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>No. Requires advanced EDR integration.</t>
+          <t>No. Our current SOAR cannot perform complex API integrations.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>SOAR playbook: live-response via EDR API</t>
+          <t>Advanced SOAR / API Integration</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -823,12 +823,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Out of Scope</t>
+          <t>Partial (Detection Only)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Shadow copy deletion detection is covered by rules AN0933, AN0602, and AN0411. However, automated rollback of encrypted files and canary file detonation are out of scope. Our SIEM is a passive log analysis engine. We lack the advanced EDR integration required for host isolation and file rollback.</t>
+          <t>Shadow copy deletion detection (a key ransomware indicator) is fully covered by rules AN0933-T1490-DET0329, AN0602-T1486-DET0215, and AN0411-T1485-DET0146. However, automated rollback of encrypted files and canary file detonation are out of scope. Our SIEM is a passive log analysis engine; physically restoring encrypted files and deploying deception decoys are active capabilities that fundamentally require a dedicated EDR agent. Real-time response requires complex API integrations which our current SOAR cannot perform.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Yes, via SOAR playbook calling EDR API.</t>
+          <t>No. Our current SOAR cannot perform complex API integrations.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>SOAR playbook: isolate-host-and-restore-files via EDR API</t>
+          <t>Advanced SOAR / API Integration</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -853,12 +853,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Basic script obfuscation checks are strongly covered by over 100 rules. However, to catch advanced scripts that hide themselves, we need Windows Event ID 1116/1117 (AMSI logs). Without IT turning on Script Block Logging via Group Policy (GPO), the SIEM is completely blind to advanced fileless scripts.</t>
+          <t>Basic script obfuscation checks (like hackers hiding commands with caret ^ symbols) are strongly covered by over 100 rules (e.g., AN1501-T1055.013-DET0544). However, our major gap is runtime deobfuscation. To catch advanced scripts that hide themselves, we desperately need Windows Event ID 1116/1117 (AMSI logs). This specific log gives us the clean, readable script content (ScriptBlockText) right before it executes. Without IT turning on 'Script Block Logging' via Group Policy (GPO), the SIEM is completely blind to advanced fileless scripts. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -967,12 +967,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Windows AMSI / Script Block Logging</t>
+          <t>Windows AMSI / EDR Platform</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Detecting data being copied to USB drives is covered by rules AN0616 and AN0342. However, to reliably log physical USB insertions, we need Windows Event ID 2003 enabled. Actively blocking USB drives or enforcing read-only policies is out of scope, as it requires a dedicated EDR or DLP agent.</t>
+          <t>Detecting data being copied to USB drives via command-line heuristics is covered by rules AN0616-T1052.001-DET0220 and AN0342-T1052-DET0123. However, we have a gap in deterministic hardware auditing; to reliably log physical USB insertions, we need Windows Event ID 2003 (DriverFrameworks-UserMode) enabled. Finally, actively blocking USB drives or enforcing read-only policies are out of scope. A SIEM cannot physically block hardware from mounting; this requires a dedicated EDR or DLP device control agent. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Tooling / Capability Gap</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1071,12 +1071,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Out of Scope</t>
+          <t>Partial (Detection Only)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Real-time blocking of malicious SHA-256 hashes and enforcing custom hash execution policies is out of scope. While our SIEM can alert on known bad hashes post-execution, physically blocking the file from executing pre-execution requires advanced EDR integration which we do not possess.</t>
+          <t>Real-time blocking of malicious SHA-256 hashes and enforcing custom hash execution policies are active response features that require a dedicated EDR agent. While our SIEM can theoretically alert on known bad hashes after they run, physically blocking the file from executing in the first place is out of scope for a passive correlation engine. Real-time response requires complex API integrations which our current SOAR cannot perform.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No. Requires advanced EDR integration.</t>
+          <t>No. Our current SOAR cannot perform complex API integrations.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>SOAR playbook: block-hash/IOC via EDR/TIP API</t>
+          <t>Advanced SOAR / API Integration</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1133,12 +1133,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Detecting attempts to kill security agents via command-line tools (like using taskkill or net stop) is covered by rules like AN0061-T1489-DET0021 and AN1369-T1685-DET0497. However, our gap is deterministic service auditing; to know for sure if a service was successfully stopped, we need Windows Event ID 7040 (Service Control Manager logs). Finally, actively protecting the agent from being uninstalled or tampered with at the kernel level is out of scope. A SIEM cannot self-protect endpoints; this requires an EDR agent with built-in anti-tamper mechanisms.</t>
+          <t>Detecting attempts to kill security agents via command-line tools (like using taskkill or net stop) is covered by rules like AN0061-T1489-DET0021 and AN1369-T1685-DET0497. However, our gap is deterministic service auditing; to know for sure if a service was successfully stopped, we need Windows Event ID 7040 (Service Control Manager logs). Finally, actively protecting the agent from being uninstalled or tampered with at the kernel level is out of scope. A SIEM cannot self-protect endpoints; this requires an EDR agent with built-in anti-tamper mechanisms. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1153,22 +1153,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Windows Event ID 7040 / EDR Platform (for protection)</t>
+          <t>EDR Platform</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Rule</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1203,11 +1203,7 @@
           <t>Providing protection while an endpoint is completely offline requires an agent running locally on the machine with its own built-in ML models and cached policies. Because a SIEM relies 100% on centralized log forwarding over the network, it is physically impossible for the correlation engine to analyze events or protect a machine during an internet outage. This is a fundamental architectural requirement for a local EDR agent.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>No. Offline ML models and caching are EDR sensor features.</t>
@@ -1257,7 +1253,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fully Covered</t>
+          <t>Covered</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1282,7 +1278,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Fully Covered</t>
+          <t>Covered</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1319,12 +1315,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Privileged process monitoring on Windows servers (like IIS and SQL) is strongly covered by over 30 rules (e.g., AN0219-T1190-DET0080). However, we have a critical gap in Linux and container visibility. To detect server attacks on Linux workloads, we absolutely need native telemetry like Auditd, Syslog, or Sysmon for Linux. For container visibility, we need logs from tools like Falco or Kubernetes audit logs. Without these specific log sources forwarding to the SIEM, we are completely blind to Linux and container compromises.</t>
+          <t>Privileged process monitoring on Windows servers (like IIS and SQL) is strongly covered by over 30 rules (e.g., AN0219-T1190-DET0080). However, we have a critical gap in Linux and container visibility. To detect server attacks on Linux workloads, we absolutely need native telemetry like Auditd, Syslog, or Sysmon for Linux. For container visibility, we need logs from tools like Falco or Kubernetes audit logs. Without these specific log sources forwarding to the SIEM, we are completely blind to Linux and container compromises. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1344,7 +1340,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1381,12 +1377,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Detecting attempts to read LSASS memory (e.g., Mimikatz dumping passwords) is strongly covered by over 20 rules (e.g., AN0235-T1003.002-DET0085). However, we have a gap for advanced identity attacks: to detect DCSync, we need Windows Event ID 4662 (Directory Service Access) capturing specific replication GUIDs. To detect NTLM relays, we need Windows Event 4624 (Logon) capturing NTLM authentication details. Finally, actively blocking these attacks is out of scope. A SIEM cannot enforce OS-level memory protections like Credential Guard or physically block network authentication relays.</t>
+          <t>Detecting attempts to read LSASS memory (e.g., Mimikatz dumping passwords) is strongly covered by over 20 rules (e.g., AN0235-T1003.002-DET0085). However, we have a gap for advanced identity attacks: to detect DCSync, we need Windows Event ID 4662 (Directory Service Access) capturing specific replication GUIDs. To detect NTLM relays, we need Windows Event 4624 (Logon) capturing NTLM authentication details. Finally, actively blocking these attacks is out of scope. A SIEM cannot enforce OS-level memory protections like Credential Guard or physically block network authentication relays. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1401,22 +1397,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Windows Event 4662 / 4624</t>
+          <t>EDR Platform</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Rule</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1439,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1463,12 +1459,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Windows Event 4703 / Linux Auditd</t>
+          <t>EDR Platform / SIEM</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1505,7 +1501,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1525,12 +1521,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Azure AD Sign-in and Audit Logs</t>
+          <t>ITDR Platform</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1572,7 +1568,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Actively enforcing Conditional Access policies, triggering MFA prompts, and checking device posture are active capabilities that require a dedicated Identity Provider (like Entra ID or Okta). A SIEM cannot physically enforce logins or block sessions in real-time. While we could theoretically audit session token theft (which is currently a log gap requiring Azure AD Sign-in Logs), the core enforcement mandate of this category is completely out of scope for a passive correlation engine.</t>
+          <t>Actively enforcing Conditional Access policies, triggering MFA prompts, and checking device posture are active capabilities that require a dedicated Identity Provider (like Entra ID or Okta). A SIEM cannot physically enforce logins or block sessions in real-time. While we could theoretically audit 'session token theft' (which is currently a log gap requiring Azure AD Sign-in Logs), the core enforcement mandate of this category is completely out of scope for a passive correlation engine. Once detection is closed (via missing log), response is separately solvable via SOAR playbook + IAM/IdP (e.g., Entra ID/Okta) API, once integrated.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1592,12 +1588,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1629,7 +1625,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1691,7 +1687,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1716,7 +1712,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1753,12 +1749,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Behavioral beacon detection and periodic communication analysis using Zeek, Suricata, and endpoint telemetry are fully covered by over 20 correlation rules (e.g., AN8002-T1071-DET8002, AN0637-T1104-DET0228). However, we have an architectural gap regarding advanced network capabilities: full DGA (Domain Generation Algorithm) classification, encrypted HTTPS payload decryption, and TLS fingerprinting are out of scope. A SIEM cannot decrypt live network traffic or perform deep packet inspection. This requires a dedicated Network Detection and Response (NDR) platform.</t>
+          <t>Behavioral beacon detection and periodic communication analysis using Zeek, Suricata, and endpoint telemetry are fully covered by over 20 correlation rules (e.g., AN8002-T1071-DET8002, AN0637-T1104-DET0228). However, we have an architectural gap regarding advanced network capabilities: full DGA (Domain Generation Algorithm) classification, encrypted HTTPS payload decryption, and TLS fingerprinting are out of scope. A SIEM cannot decrypt live network traffic or perform deep packet inspection. This requires a dedicated Network Detection and Response (NDR) platform. Importantly, because we have active Threat Intel feeds, we successfully detect and use our SOAR to block known bad C2 IPs and domains. The remaining gap is strictly for advanced unknown/zero-day encrypted payloads and dynamic DGA.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1768,12 +1764,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Sigma alone is weak for this. Best addressed via NDR or Threat Intel feeds + frequency analysis as a stopgap.</t>
+          <t>Yes for known threats (using our existing Threat Intel feeds). Unknown/encrypted C2s still require an NDR.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>NDR Platform / EDR Platform</t>
+          <t>NDR Platform (only for unknown/encrypted C2)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1815,7 +1811,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fully Covered</t>
+          <t>Covered</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1835,12 +1831,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>N/A (Covered by existing Windows Event Logs)</t>
+          <t>EDR Platform / NDR Platform</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Fully Covered</t>
+          <t>Covered</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1877,7 +1873,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1939,7 +1935,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2006,7 +2002,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Actively blocking malicious domains (sinkholing) and preventing DNS-based exfiltration in real-time are out of scope. A SIEM is a passive log analyzer; it cannot physically intercept or block DNS requests. This requires a dedicated DNS security platform (like Cisco Umbrella) or a Next-Gen Firewall. Furthermore, we currently have a log gap for detecting advanced DNS threats: to alert on DNS-over-HTTPS (DoH) or recursive anomalies, we need dedicated DNS infrastructure telemetry (like Windows DNS Server Analytical logs or Zeek DNS logs).</t>
+          <t>Actively blocking malicious domains (sinkholing) and preventing DNS-based exfiltration in real-time are out of scope. A SIEM is a passive log analyzer; it cannot physically intercept or block DNS requests. This requires a dedicated DNS security platform (like Cisco Umbrella) or a Next-Gen Firewall. Furthermore, we currently have a log gap for detecting advanced DNS threats: to alert on DNS-over-HTTPS (DoH) or recursive anomalies, we need dedicated DNS infrastructure telemetry (like Windows DNS Server Analytical logs or Zeek DNS logs). Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2026,12 +2022,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2125,7 +2121,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2150,7 +2146,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2257,11 +2253,7 @@
           <t>Proxying email links through a reputation engine and actively rewriting URLs for time-of-click protection are entirely out of scope. A SIEM is a passive analytics platform that analyzes logs after an event occurs; it does not sit inline with email delivery routing. Therefore, it cannot physically intercept, rewrite, or proxy email URLs. This capability requires a dedicated Secure Email Gateway (like Proofpoint TAP or Mimecast).</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>No. Time-of-click protection is an Email Gateway feature.</t>
@@ -2316,7 +2308,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Actively enforcing email authentication policies (like dropping emails that fail DMARC/SPF checks) and blocking spoofed domains are completely out of scope. A SIEM is a passive log analyzer; it cannot physically drop inbound emails or publish outbound DNS policies. This enforcement must happen at the Secure Email Gateway (SEG) layer (e.g., Proofpoint, O365). While we could theoretically alert on authentication failures, that is currently a log gap because we lack the email header logs to do so.</t>
+          <t>Actively enforcing email authentication policies (like dropping emails that fail DMARC/SPF checks) and blocking spoofed domains are completely out of scope. A SIEM is a passive log analyzer; it cannot physically drop inbound emails or publish outbound DNS policies. This enforcement must happen at the Secure Email Gateway (SEG) layer (e.g., Proofpoint, O365). While we could theoretically alert on authentication failures, that is currently a log gap because we lack the email header logs to do so. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2336,12 +2328,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2381,11 +2373,7 @@
           <t>Analyzing the natural language of an email body to detect 'urgent payment requests' or 'anomalous bank details' is completely out of scope. A SIEM is a structured log search engine; it cannot run Natural Language Processing (NLP) or AI models against the unstructured text of an email body. This deep semantic analysis physically requires a specialized API-based email security platform (like Abnormal Security or Tessian).</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>No. Requires ML-based email security.</t>
@@ -2435,7 +2423,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2460,7 +2448,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Telemetry / Log Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2502,7 +2490,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Actively blocking the exfiltration of classified documents and enforcing sensitivity labels on outbound emails are completely out of scope. A SIEM is a passive analytics platform; it cannot inspect email body content mid-flight or physically block an email from leaving the network. These capabilities require a dedicated Data Loss Prevention (DLP) solution (like Microsoft Purview). While we could theoretically alert on bulk external recipients, this is currently a log gap because we lack Office 365 Message Trace logs.</t>
+          <t>Actively blocking the exfiltration of classified documents and enforcing sensitivity labels on outbound emails are completely out of scope. A SIEM is a passive analytics platform; it cannot inspect email body content mid-flight or physically block an email from leaving the network. These capabilities require a dedicated Data Loss Prevention (DLP) solution (like Microsoft Purview). While we could theoretically alert on bulk external recipients, this is currently a log gap because we lack Office 365 Message Trace logs. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2522,12 +2510,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2621,7 +2609,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2708,7 +2696,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Tooling / Capability Gap</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2718,7 +2706,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2869,12 +2857,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Detecting basic insider sabotage (like using command-line tools for mass file deletion or clearing event logs) is fully covered by our correlation rules (e.g., AN0411-T1485-DET0146). However, we have a significant capability gap regarding stateful User Behavior Analytics (UEBA). Sigma correlation rules are stateless queries; they cannot dynamically baseline a user's normal working hours to trigger 'after-hours anomalies' or 'resignation patterns'. Additionally, detecting mass cloud downloads is a log gap that requires Office 365 Audit logs.</t>
+          <t>Detecting basic insider sabotage (like using command-line tools for mass file deletion or clearing event logs) is fully covered by our correlation rules (e.g., AN0411-T1485-DET0146). However, we have a significant capability gap regarding long-term User Behavior Analytics (UEBA). Our correlation rules only look for specific predefined patterns in logs; they cannot build long-term historical profiles (like a user's normal working hours over a month) to flag unusual deviations like 'after-hours anomalies' or 'resignation patterns'. Additionally, detecting mass cloud downloads is a log gap that requires Office 365 Audit logs.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2884,7 +2872,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>No. Sigma evaluates single events statelessly; it cannot do UEBA.</t>
+          <t>No. The rule engine evaluates logs for specific immediate patterns; it cannot build long-term user behavior profiles (UEBA).</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2894,7 +2882,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Tooling / Capability Gap</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2904,14 +2892,14 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Emerging Ai</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2939,11 +2927,7 @@
           <t>Running predictive Machine Learning (ML) models on the endpoint to score attack chains and predict zero-days is completely out of scope. Sigma rules are deterministic, logic-based queries (signatures and heuristics). They cannot train or execute AI/ML models on a host. This capability physically requires a Next-Gen Antivirus (NGAV) or an EDR agent with built-in ML sensors.</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>No. Predictive ML is an EDR feature.</t>
@@ -2998,14 +2982,10 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Actively blocking AI bots, inspecting data submitted to LLMs (like ChatGPT or Copilot) for DLP, and detecting prompt injections in real-time are completely out of scope. A SIEM cannot intercept web sessions to read or block chat prompts. This capability physically requires a Cloud Access Security Broker (CASB) or a dedicated GenAI Security Gateway. While we could theoretically audit AI website visits, this remains a log gap because we lack Proxy/SWG traffic logs.</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+          <t>Actively blocking AI bots, inspecting data submitted to LLMs (like ChatGPT or Copilot) for DLP, and detecting prompt injections in real-time are completely out of scope. A SIEM cannot intercept web sessions to read or block chat prompts. This capability physically requires a Cloud Access Security Broker (CASB) or a dedicated GenAI Security Gateway. While we could theoretically audit AI website visits, this remains a log gap because we lack Proxy/SWG traffic logs. Even if detection is solved, complex response actions via external APIs are beyond our current SOAR capabilities.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>No. Requires a CASB or Secure Web Gateway.</t>
@@ -3018,12 +2998,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3063,11 +3043,7 @@
           <t>Monitoring the dark web for exposed credentials and automatically operationalising STIX/TAXII IOCs into blocking rules are completely out of scope. A SIEM is an analytics engine; it does not natively scrape the dark web or automatically orchestrate intelligence feeds for active blocking. This capability physically requires a Threat Intelligence Platform (TIP) (like ThreatConnect or MISP) integrated with a SOAR.</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>No. Requires a TIP or SOAR.</t>
@@ -3097,7 +3073,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3125,11 +3101,7 @@
           <t>Continuously scanning the external internet for exposed assets, open ports, and monitoring the dark web for leaked government credentials are completely out of scope. A SIEM is a passive log receiver; it does not proactively scan the external internet or perform vulnerability discovery. This capability physically requires a dedicated External Attack Surface Management (EASM) platform (like Microsoft Defender EASM or Cortex Xpanse).</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>No. Requires EASM scanner.</t>
@@ -3187,11 +3159,7 @@
           <t>Using AI to automatically perform root cause analysis, suppress false positives, and generate natural language incident summaries is entirely out of scope for our correlation rules. Sigma rules are static, logic-based queries; they do not possess an AI engine or automation capabilities to triage their own alerts. This requires a Security Orchestration, Automation, and Response (SOAR) tool or an AI assistant (like Microsoft Security Copilot).</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>No. Requires AI-driven SOAR.</t>
@@ -3241,19 +3209,15 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Monitoring decoy files or 'honey-token' accounts for unauthorized access is easily achievable with our SIEM by writing custom queries for specific fake usernames or file paths. However, automatically generating, deploying, and rotating these fake credentials, decoy files, and virtual honeypot servers across the enterprise is completely out of scope. That active deployment capability physically requires a dedicated Deception Technology platform (like Thinkst Canary).</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+          <t>We can detect if a hacker touches a fake file or fake account. That is fully covered. However, we cannot automatically create or deploy these fake files and accounts across the network. To actually build and spread them, you need a separate Deception tool.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>No. Requires deploying actual honeypots.</t>
@@ -3311,11 +3275,7 @@
           <t>Proactively scanning AWS/Azure APIs to detect cloud misconfigurations, mapping assets to CIS/NIST compliance frameworks, and executing auto-remediation workflows are entirely out of scope. A SIEM analyzes logs of discrete events (e.g., a user changing a setting); it does not natively query cloud control planes to audit static configuration states. This capability physically requires a Cloud Security Posture Management (CSPM) platform (like Wiz or Prisma Cloud).</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>No. Requires CSPM.</t>
@@ -3390,7 +3350,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Tooling / Capability Gap</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3400,7 +3360,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3452,12 +3412,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Tooling &amp; Telemetry Gap</t>
+          <t>Missing Logs</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3497,11 +3457,7 @@
           <t>Performing passive, agentless discovery of IoT/OT devices (like printers or SCADA systems) and dynamically enforcing network segmentation policies are completely out of scope. A SIEM analyzes structured logs; it does not passively sniff raw network traffic on the wire to fingerprint unmanaged devices. This capability physically requires a dedicated Network Detection and Response (NDR) or OT security appliance (like Claroty or Nozomi).</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>No. Requires NDR or OT scanner.</t>
@@ -3559,11 +3515,7 @@
           <t>A Cloud-Native Application Protection Platform (CNAPP) is an entire suite of proactive cloud security tools. Replacing a CNAPP is completely out of scope for a SIEM. A SIEM analyzes discrete event logs; it cannot perform infrastructure-as-code (IaC) vulnerability scanning, runtime container protection, or active cloud permissions enforcement. This physically requires a dedicated CNAPP platform (like Wiz or Prisma Cloud).</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>N/A (Architecture / Non-Atomic)</t>
-        </is>
-      </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>No. Requires CNAPP vendor.</t>

</xml_diff>